<commit_message>
label GMV, Equal weight, frontier without defense
</commit_message>
<xml_diff>
--- a/Project 1/defense_results/analysis_results.xlsx
+++ b/Project 1/defense_results/analysis_results.xlsx
@@ -17,11 +17,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exclusion_cost" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="defense_weight_sensitivity" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bootstrap_gmv_defense" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monthly_returns" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frontier_full_with_def" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_audit" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="security_history" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="periods" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="returns_test" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="question_answer" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monthly_returns" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frontier_full_with_def" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_audit" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="security_history" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="periods" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -51,7 +53,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -64,6 +66,27 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -853,6 +876,236 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Pre-invasion annualized mean</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.188482706995672</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Post-invasion annualized mean</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.09883805855208924</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Difference (post - pre), annualized</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.0896446484435828</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Standard error of difference, annualized</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.09912376354075705</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>t-statistic</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.9043709120943869</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Degrees of freedom (Welch)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>81.78186331488877</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Two-sided p-value</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3684551720365185</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Pre-invasion</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Post-invasion</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Change (post - pre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Diversification test</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Average correlation of DEF with sectors</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.5486283832502574</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.3927084394723381</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.1559199437779193</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>DEF weight in minimum variance portfolio</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.05540182866451901</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.2214304253984209</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1660285967339019</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Extra minimum-variance volatility from excluding DEF</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0002831058937632913</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.005021155056011709</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.004738049162248417</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Returns test</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>DEF annualized mean return</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.188482706995672</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.09883805855208924</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.0896446484435828</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>DEF weight in mean-variance utility portfolio (γ = 4)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.4025461561604331</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.2221693546039033</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.1803768015565298</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A2:A4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6871,7 +7124,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10525,7 +10778,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10610,7 +10863,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11084,7 +11337,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12812,7 +13065,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Utility max (A=4)</t>
+          <t>Mean-variance utility (γ=4)</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -12906,7 +13159,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Utility max (A=4)</t>
+          <t>Mean-variance utility (γ=4)</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -13000,7 +13253,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Utility max (A=4)</t>
+          <t>Mean-variance utility (γ=4)</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -13094,7 +13347,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Utility max (A=4)</t>
+          <t>Mean-variance utility (γ=4)</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -13188,7 +13441,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Utility max (A=4)</t>
+          <t>Mean-variance utility (γ=4)</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
@@ -13282,7 +13535,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Utility max (A=4)</t>
+          <t>Mean-variance utility (γ=4)</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -13491,7 +13744,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>A = 2</t>
+          <t>γ = 2</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -13507,7 +13760,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>A = 4</t>
+          <t>γ = 4</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -13523,7 +13776,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>A = 6</t>
+          <t>γ = 6</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -13539,7 +13792,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>A = 8</t>
+          <t>γ = 8</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -13555,7 +13808,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>A = 10</t>
+          <t>γ = 10</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">

</xml_diff>